<commit_message>
finished chi sq tests
</commit_message>
<xml_diff>
--- a/GMV_timing_tempo_models/SB_Chi-Square difference test.xlsx
+++ b/GMV_timing_tempo_models/SB_Chi-Square difference test.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://uvmoffice-my.sharepoint.com/personal/abrieant_uvm_edu/Documents/OneDrive/Manuscripts/reg report DCN/pubertybrain/GMV_timing_tempo_models/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="85" documentId="8_{56B60A14-3F50-8646-A359-166224E3E378}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{A81C5BA8-19C4-CF4C-B648-72CEB69299B7}"/>
+  <xr:revisionPtr revIDLastSave="148" documentId="8_{56B60A14-3F50-8646-A359-166224E3E378}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{AE47FC73-1958-3543-A6D0-8CBABCDF71B5}"/>
   <bookViews>
     <workbookView xWindow="20" yWindow="500" windowWidth="28780" windowHeight="17200" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -35,7 +35,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="22" uniqueCount="16">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="23" uniqueCount="23">
   <si>
     <t>F1</t>
   </si>
@@ -106,6 +106,27 @@
   <si>
     <t>MCORT: latent vs linear</t>
   </si>
+  <si>
+    <t>FSCORT: linear vs no growth</t>
+  </si>
+  <si>
+    <t>FSCORT: quad vs linear</t>
+  </si>
+  <si>
+    <t>FSCORT: latent vs linear</t>
+  </si>
+  <si>
+    <t>MSCORT: linear vs no growth</t>
+  </si>
+  <si>
+    <t>MSCORT: quad vs linear</t>
+  </si>
+  <si>
+    <t>MSCORT: latent vs linear</t>
+  </si>
+  <si>
+    <t>N/A</t>
+  </si>
 </sst>
 </file>
 
@@ -160,7 +181,7 @@
       <family val="1"/>
     </font>
   </fonts>
-  <fills count="3">
+  <fills count="5">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -170,6 +191,18 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor theme="2" tint="-9.9978637043366805E-2"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="3" tint="0.79998168889431442"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="6" tint="0.79998168889431442"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -186,11 +219,8 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="16">
+  <cellXfs count="28">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
@@ -202,9 +232,6 @@
     <xf numFmtId="164" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
@@ -214,16 +241,54 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="2" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="4" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="2" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="4" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="2" fontId="1" fillId="3" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="1" fillId="3" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="2" fontId="0" fillId="3" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="2" fontId="1" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="1" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -2039,355 +2104,484 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:10" ht="231.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A1" s="8"/>
-      <c r="B1" s="9"/>
-      <c r="C1" s="9"/>
-      <c r="D1" s="10"/>
-      <c r="E1" s="10"/>
-      <c r="F1" s="10"/>
-      <c r="G1" s="10"/>
-      <c r="H1" s="10"/>
-      <c r="I1" s="10"/>
-      <c r="J1" s="10"/>
+      <c r="A1" s="6"/>
+      <c r="B1" s="7"/>
+      <c r="C1" s="7"/>
+      <c r="D1" s="8"/>
+      <c r="E1" s="8"/>
+      <c r="F1" s="8"/>
+      <c r="G1" s="8"/>
+      <c r="H1" s="8"/>
+      <c r="I1" s="8"/>
+      <c r="J1" s="8"/>
     </row>
     <row r="2" spans="1:10" x14ac:dyDescent="0.2">
-      <c r="A2" s="3"/>
-      <c r="B2" s="4" t="s">
+      <c r="A2" s="2"/>
+      <c r="B2" s="3" t="s">
         <v>2</v>
       </c>
-      <c r="C2" s="4" t="s">
+      <c r="C2" s="3" t="s">
         <v>3</v>
       </c>
-      <c r="D2" s="4" t="s">
+      <c r="D2" s="3" t="s">
         <v>4</v>
       </c>
-      <c r="E2" s="4" t="s">
+      <c r="E2" s="3" t="s">
         <v>5</v>
       </c>
-      <c r="F2" s="4" t="s">
+      <c r="F2" s="3" t="s">
         <v>0</v>
       </c>
-      <c r="G2" s="4" t="s">
+      <c r="G2" s="3" t="s">
         <v>1</v>
       </c>
-      <c r="H2" s="4" t="s">
+      <c r="H2" s="3" t="s">
         <v>6</v>
       </c>
-      <c r="I2" s="4" t="s">
+      <c r="I2" s="3" t="s">
         <v>7</v>
       </c>
-      <c r="J2" s="4" t="s">
+      <c r="J2" s="3" t="s">
         <v>8</v>
       </c>
     </row>
     <row r="3" spans="1:10" x14ac:dyDescent="0.2">
-      <c r="A3" s="5" t="s">
+      <c r="A3" s="4" t="s">
         <v>9</v>
       </c>
-      <c r="B3" s="2">
+      <c r="B3" s="10">
         <v>0.95799999999999996</v>
       </c>
-      <c r="C3" s="2">
+      <c r="C3" s="10">
         <v>1.018</v>
       </c>
-      <c r="D3" s="2">
+      <c r="D3" s="1">
         <v>6</v>
       </c>
-      <c r="E3" s="2">
+      <c r="E3" s="1">
         <v>8</v>
       </c>
-      <c r="F3" s="2">
+      <c r="F3" s="1">
         <v>35.122</v>
       </c>
-      <c r="G3" s="2">
+      <c r="G3" s="1">
         <v>178.09700000000001</v>
       </c>
-      <c r="H3" s="12">
+      <c r="H3" s="9">
         <f t="shared" ref="H3" si="0">(G3*C3-F3*B3)*(E3-D3)/(C3*E3-B3*D3)</f>
         <v>123.25197829716191</v>
       </c>
-      <c r="I3" s="2">
+      <c r="I3" s="1">
         <f t="shared" ref="I3:I5" si="1">E3-D3</f>
         <v>2</v>
       </c>
-      <c r="J3" s="6">
+      <c r="J3" s="5">
         <f t="shared" ref="J3:J5" si="2">_xlfn.CHISQ.DIST.RT(H3,I3)</f>
         <v>1.7225544979244626E-27</v>
       </c>
     </row>
-    <row r="4" spans="1:10" ht="16" x14ac:dyDescent="0.2">
-      <c r="A4" t="s">
+    <row r="4" spans="1:10" s="11" customFormat="1" ht="16" x14ac:dyDescent="0.2">
+      <c r="A4" s="11" t="s">
         <v>10</v>
       </c>
-      <c r="B4" s="14">
+      <c r="B4" s="12">
         <v>1.99</v>
       </c>
-      <c r="C4" s="14">
+      <c r="C4" s="12">
         <v>2.0699999999999998</v>
       </c>
-      <c r="D4" s="1">
+      <c r="D4" s="13">
         <v>8</v>
       </c>
-      <c r="E4" s="1">
+      <c r="E4" s="13">
         <v>11</v>
       </c>
-      <c r="F4" s="11">
+      <c r="F4" s="14">
         <v>317.69</v>
       </c>
-      <c r="G4" s="11">
+      <c r="G4" s="14">
         <v>4817.8900000000003</v>
       </c>
-      <c r="H4" s="12">
+      <c r="H4" s="15">
         <f>(G4*C4-F4*B4)*(E4-D4)/(C4*E4-B4*D4)</f>
         <v>4090.8741021897813</v>
       </c>
-      <c r="I4" s="2">
+      <c r="I4" s="16">
         <f t="shared" si="1"/>
         <v>3</v>
       </c>
-      <c r="J4" s="6">
+      <c r="J4" s="17">
         <f t="shared" si="2"/>
         <v>0</v>
       </c>
     </row>
-    <row r="5" spans="1:10" ht="16" x14ac:dyDescent="0.2">
-      <c r="A5" s="7" t="s">
+    <row r="5" spans="1:10" s="11" customFormat="1" ht="16" x14ac:dyDescent="0.2">
+      <c r="A5" s="18" t="s">
         <v>11</v>
       </c>
-      <c r="B5" s="1">
+      <c r="B5" s="19">
         <v>2.09</v>
       </c>
-      <c r="C5" s="1">
+      <c r="C5" s="19">
         <v>1.99</v>
       </c>
-      <c r="D5" s="1">
+      <c r="D5" s="13">
         <v>7</v>
       </c>
-      <c r="E5" s="1">
+      <c r="E5" s="13">
         <v>8</v>
       </c>
-      <c r="F5" s="11">
+      <c r="F5" s="14">
         <v>236.11</v>
       </c>
-      <c r="G5" s="1">
+      <c r="G5" s="13">
         <f>F4</f>
         <v>317.69</v>
       </c>
-      <c r="H5" s="12">
+      <c r="H5" s="15">
         <f>(G5*C5-F5*B5)*(E5-D5)/(C5*E5-B5*D5)</f>
         <v>107.54511627906966</v>
       </c>
-      <c r="I5" s="2">
+      <c r="I5" s="16">
         <f t="shared" si="1"/>
         <v>1</v>
       </c>
-      <c r="J5" s="6">
+      <c r="J5" s="17">
         <f t="shared" si="2"/>
         <v>3.381201200735192E-25</v>
       </c>
     </row>
-    <row r="6" spans="1:10" ht="16" x14ac:dyDescent="0.2">
-      <c r="A6" s="7" t="s">
+    <row r="6" spans="1:10" s="11" customFormat="1" ht="16" x14ac:dyDescent="0.2">
+      <c r="A6" s="18" t="s">
         <v>14</v>
       </c>
-      <c r="B6" s="1">
+      <c r="B6" s="19">
         <v>2</v>
       </c>
-      <c r="C6" s="1">
+      <c r="C6" s="19">
         <v>1.99</v>
       </c>
-      <c r="D6" s="1">
+      <c r="D6" s="13">
         <v>6</v>
       </c>
-      <c r="E6" s="1">
+      <c r="E6" s="13">
         <v>8</v>
       </c>
-      <c r="F6" s="13">
+      <c r="F6" s="20">
         <v>79.540000000000006</v>
       </c>
-      <c r="G6" s="1">
+      <c r="G6" s="13">
         <f>F5</f>
         <v>236.11</v>
       </c>
-      <c r="H6" s="12">
+      <c r="H6" s="15">
         <f t="shared" ref="H6:H11" si="3">(G6*C6-F6*B6)*(E6-D6)/(C6*E6-B6*D6)</f>
         <v>158.56066326530615</v>
       </c>
-      <c r="I6" s="2">
+      <c r="I6" s="16">
         <f t="shared" ref="I6" si="4">E6-D6</f>
         <v>2</v>
       </c>
-      <c r="J6" s="6">
+      <c r="J6" s="17">
         <f t="shared" ref="J6" si="5">_xlfn.CHISQ.DIST.RT(H6,I6)</f>
         <v>3.7067171591653342E-35</v>
       </c>
     </row>
-    <row r="7" spans="1:10" ht="16" x14ac:dyDescent="0.2">
-      <c r="A7" t="s">
+    <row r="7" spans="1:10" s="11" customFormat="1" ht="16" x14ac:dyDescent="0.2">
+      <c r="A7" s="11" t="s">
         <v>12</v>
       </c>
-      <c r="B7" s="11">
+      <c r="B7" s="12">
         <v>2.25</v>
       </c>
-      <c r="C7" s="11">
+      <c r="C7" s="12">
         <v>2.38</v>
       </c>
-      <c r="D7" s="1">
+      <c r="D7" s="13">
         <v>8</v>
       </c>
-      <c r="E7" s="1">
+      <c r="E7" s="13">
         <v>11</v>
       </c>
-      <c r="F7" s="11">
+      <c r="F7" s="14">
         <v>142.22999999999999</v>
       </c>
-      <c r="G7" s="11">
+      <c r="G7" s="14">
         <v>2889.44</v>
       </c>
-      <c r="H7" s="12">
+      <c r="H7" s="15">
         <f t="shared" si="3"/>
         <v>2404.7126039119808</v>
       </c>
-      <c r="I7" s="2">
+      <c r="I7" s="16">
         <f>E7-D7</f>
         <v>3</v>
       </c>
-      <c r="J7" s="6">
+      <c r="J7" s="17">
         <f>_xlfn.CHISQ.DIST.RT(H7,I7)</f>
         <v>0</v>
       </c>
     </row>
-    <row r="8" spans="1:10" x14ac:dyDescent="0.2">
-      <c r="A8" s="7" t="s">
+    <row r="8" spans="1:10" s="11" customFormat="1" x14ac:dyDescent="0.2">
+      <c r="A8" s="18" t="s">
         <v>13</v>
       </c>
-      <c r="B8" s="15">
+      <c r="B8" s="21">
         <v>2.4900000000000002</v>
       </c>
-      <c r="C8" s="1">
+      <c r="C8" s="19">
         <v>2.25</v>
       </c>
-      <c r="D8" s="1">
+      <c r="D8" s="13">
         <v>4</v>
       </c>
-      <c r="E8" s="1">
+      <c r="E8" s="13">
         <v>8</v>
       </c>
-      <c r="F8" s="1">
+      <c r="F8" s="13">
         <v>31.62</v>
       </c>
-      <c r="G8" s="1">
+      <c r="G8" s="13">
         <v>142.22999999999999</v>
       </c>
-      <c r="H8" s="12">
+      <c r="H8" s="15">
         <f t="shared" si="3"/>
         <v>120.04164179104478</v>
       </c>
-      <c r="I8" s="2">
+      <c r="I8" s="16">
         <f>E8-D8</f>
         <v>4</v>
       </c>
-      <c r="J8" s="6">
+      <c r="J8" s="17">
         <f>_xlfn.CHISQ.DIST.RT(H8,I8)</f>
         <v>5.2331927560267366E-25</v>
       </c>
     </row>
-    <row r="9" spans="1:10" ht="16" x14ac:dyDescent="0.2">
-      <c r="A9" s="7" t="s">
+    <row r="9" spans="1:10" s="11" customFormat="1" ht="16" x14ac:dyDescent="0.2">
+      <c r="A9" s="18" t="s">
         <v>15</v>
       </c>
-      <c r="B9">
+      <c r="B9" s="19">
         <v>2.5</v>
       </c>
-      <c r="C9" s="1">
+      <c r="C9" s="19">
         <v>2.25</v>
       </c>
-      <c r="D9" s="1">
+      <c r="D9" s="13">
         <v>6</v>
       </c>
-      <c r="E9" s="1">
+      <c r="E9" s="13">
         <v>8</v>
       </c>
-      <c r="F9" s="11">
+      <c r="F9" s="14">
         <v>36.299999999999997</v>
       </c>
-      <c r="G9" s="1">
+      <c r="G9" s="13">
         <v>142.22999999999999</v>
       </c>
-      <c r="H9" s="12">
+      <c r="H9" s="15">
         <f t="shared" si="3"/>
         <v>152.845</v>
       </c>
-      <c r="I9" s="2">
+      <c r="I9" s="16">
         <f t="shared" ref="I9:I11" si="6">E9-D9</f>
         <v>2</v>
       </c>
-      <c r="J9" s="6">
+      <c r="J9" s="17">
         <f t="shared" ref="J9:J11" si="7">_xlfn.CHISQ.DIST.RT(H9,I9)</f>
         <v>6.4584746123814661E-34</v>
       </c>
     </row>
-    <row r="10" spans="1:10" x14ac:dyDescent="0.2">
-      <c r="A10" t="s">
-        <v>10</v>
-      </c>
-      <c r="B10" s="1"/>
-      <c r="C10" s="1"/>
-      <c r="E10" s="1"/>
-      <c r="F10" s="1"/>
-      <c r="G10" s="1"/>
-      <c r="H10" s="12" t="e">
-        <f t="shared" si="3"/>
+    <row r="10" spans="1:10" s="22" customFormat="1" x14ac:dyDescent="0.2">
+      <c r="A10" s="22" t="s">
+        <v>16</v>
+      </c>
+      <c r="B10" s="23">
+        <v>3.06</v>
+      </c>
+      <c r="C10" s="23">
+        <v>2.67</v>
+      </c>
+      <c r="D10" s="23">
+        <v>8</v>
+      </c>
+      <c r="E10" s="23">
+        <v>11</v>
+      </c>
+      <c r="F10" s="23">
+        <v>346.93</v>
+      </c>
+      <c r="G10" s="23">
+        <v>452.59</v>
+      </c>
+      <c r="H10" s="24">
+        <f t="shared" si="3"/>
+        <v>90.067177914110388</v>
+      </c>
+      <c r="I10" s="25">
+        <f t="shared" si="6"/>
+        <v>3</v>
+      </c>
+      <c r="J10" s="26">
+        <f t="shared" si="7"/>
+        <v>2.1189865438803027E-19</v>
+      </c>
+    </row>
+    <row r="11" spans="1:10" s="22" customFormat="1" x14ac:dyDescent="0.2">
+      <c r="A11" s="27" t="s">
+        <v>17</v>
+      </c>
+      <c r="B11" s="23">
+        <v>2.83</v>
+      </c>
+      <c r="C11" s="23">
+        <v>3.06</v>
+      </c>
+      <c r="D11" s="23">
+        <v>7</v>
+      </c>
+      <c r="E11" s="23">
+        <v>8</v>
+      </c>
+      <c r="F11" s="23">
+        <v>117.59</v>
+      </c>
+      <c r="G11" s="23">
+        <v>346.93</v>
+      </c>
+      <c r="H11" s="24">
+        <f t="shared" si="3"/>
+        <v>156.06554603854397</v>
+      </c>
+      <c r="I11" s="25">
+        <f t="shared" si="6"/>
+        <v>1</v>
+      </c>
+      <c r="J11" s="26">
+        <f t="shared" si="7"/>
+        <v>8.1911385630297703E-36</v>
+      </c>
+    </row>
+    <row r="12" spans="1:10" s="22" customFormat="1" x14ac:dyDescent="0.2">
+      <c r="A12" s="27" t="s">
+        <v>18</v>
+      </c>
+      <c r="B12" s="23" t="s">
+        <v>22</v>
+      </c>
+      <c r="C12" s="23"/>
+      <c r="D12" s="23"/>
+      <c r="E12" s="23"/>
+      <c r="F12" s="23"/>
+      <c r="G12" s="23"/>
+      <c r="H12" s="24" t="e">
+        <f t="shared" ref="H12:H15" si="8">(G12*C12-F12*B12)*(E12-D12)/(C12*E12-B12*D12)</f>
+        <v>#VALUE!</v>
+      </c>
+      <c r="I12" s="25">
+        <f t="shared" ref="I12:I15" si="9">E12-D12</f>
+        <v>0</v>
+      </c>
+      <c r="J12" s="26" t="e">
+        <f t="shared" ref="J12:J15" si="10">_xlfn.CHISQ.DIST.RT(H12,I12)</f>
+        <v>#VALUE!</v>
+      </c>
+    </row>
+    <row r="13" spans="1:10" s="22" customFormat="1" x14ac:dyDescent="0.2">
+      <c r="A13" s="22" t="s">
+        <v>19</v>
+      </c>
+      <c r="B13" s="23">
+        <v>3.32</v>
+      </c>
+      <c r="C13" s="23">
+        <v>3.42</v>
+      </c>
+      <c r="D13" s="23">
+        <v>8</v>
+      </c>
+      <c r="E13" s="23">
+        <v>11</v>
+      </c>
+      <c r="F13" s="23">
+        <v>171.89</v>
+      </c>
+      <c r="G13" s="23">
+        <v>1283.3900000000001</v>
+      </c>
+      <c r="H13" s="24">
+        <f t="shared" si="8"/>
+        <v>1035.7646473779387</v>
+      </c>
+      <c r="I13" s="25">
+        <f t="shared" si="9"/>
+        <v>3</v>
+      </c>
+      <c r="J13" s="26">
+        <f t="shared" si="10"/>
+        <v>3.1372840592862073E-224</v>
+      </c>
+    </row>
+    <row r="14" spans="1:10" s="22" customFormat="1" x14ac:dyDescent="0.2">
+      <c r="A14" s="27" t="s">
+        <v>20</v>
+      </c>
+      <c r="B14" s="23">
+        <v>3.4</v>
+      </c>
+      <c r="C14" s="23">
+        <v>3.32</v>
+      </c>
+      <c r="D14" s="23">
+        <v>7</v>
+      </c>
+      <c r="E14" s="23">
+        <v>8</v>
+      </c>
+      <c r="F14" s="23">
+        <v>73.98</v>
+      </c>
+      <c r="G14" s="23">
+        <v>171.89</v>
+      </c>
+      <c r="H14" s="24">
+        <f t="shared" si="8"/>
+        <v>115.63144927536234</v>
+      </c>
+      <c r="I14" s="25">
+        <f t="shared" si="9"/>
+        <v>1</v>
+      </c>
+      <c r="J14" s="26">
+        <f t="shared" si="10"/>
+        <v>5.723662087760879E-27</v>
+      </c>
+    </row>
+    <row r="15" spans="1:10" s="22" customFormat="1" x14ac:dyDescent="0.2">
+      <c r="A15" s="27" t="s">
+        <v>21</v>
+      </c>
+      <c r="B15" s="23"/>
+      <c r="C15" s="23"/>
+      <c r="D15" s="23">
+        <v>6</v>
+      </c>
+      <c r="E15" s="23">
+        <v>8</v>
+      </c>
+      <c r="F15" s="23"/>
+      <c r="G15" s="23"/>
+      <c r="H15" s="24" t="e">
+        <f t="shared" si="8"/>
         <v>#DIV/0!</v>
       </c>
-      <c r="I10" s="2">
-        <f t="shared" si="6"/>
-        <v>0</v>
-      </c>
-      <c r="J10" s="6" t="e">
-        <f t="shared" si="7"/>
+      <c r="I15" s="25">
+        <f t="shared" si="9"/>
+        <v>2</v>
+      </c>
+      <c r="J15" s="26" t="e">
+        <f t="shared" si="10"/>
         <v>#DIV/0!</v>
-      </c>
-    </row>
-    <row r="11" spans="1:10" x14ac:dyDescent="0.2">
-      <c r="A11" s="7" t="s">
-        <v>11</v>
-      </c>
-      <c r="B11" s="1"/>
-      <c r="C11" s="1"/>
-      <c r="E11" s="1"/>
-      <c r="G11" s="1"/>
-      <c r="H11" s="12" t="e">
-        <f t="shared" si="3"/>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="I11" s="2">
-        <f t="shared" si="6"/>
-        <v>0</v>
-      </c>
-      <c r="J11" s="6" t="e">
-        <f t="shared" si="7"/>
-        <v>#DIV/0!</v>
-      </c>
-    </row>
-    <row r="12" spans="1:10" x14ac:dyDescent="0.2">
-      <c r="A12" s="7" t="s">
-        <v>14</v>
-      </c>
-    </row>
-    <row r="13" spans="1:10" x14ac:dyDescent="0.2">
-      <c r="A13" t="s">
-        <v>12</v>
-      </c>
-    </row>
-    <row r="14" spans="1:10" x14ac:dyDescent="0.2">
-      <c r="A14" s="7" t="s">
-        <v>13</v>
-      </c>
-    </row>
-    <row r="15" spans="1:10" x14ac:dyDescent="0.2">
-      <c r="A15" s="7" t="s">
-        <v>15</v>
       </c>
     </row>
   </sheetData>
@@ -2407,24 +2601,24 @@
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <sheetData>
     <row r="1" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="B1" s="2">
+      <c r="B1" s="1">
         <v>0.1</v>
       </c>
-      <c r="C1" s="2">
+      <c r="C1" s="1">
         <v>0.05</v>
       </c>
-      <c r="D1" s="2">
+      <c r="D1" s="1">
         <v>2.5000000000000001E-2</v>
       </c>
-      <c r="E1" s="2">
+      <c r="E1" s="1">
         <v>0.01</v>
       </c>
-      <c r="F1" s="2">
+      <c r="F1" s="1">
         <v>1E-3</v>
       </c>
     </row>
     <row r="2" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="A2" s="2">
+      <c r="A2" s="1">
         <v>1</v>
       </c>
       <c r="B2">
@@ -2449,7 +2643,7 @@
       </c>
     </row>
     <row r="3" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="A3" s="2">
+      <c r="A3" s="1">
         <v>2</v>
       </c>
       <c r="B3">
@@ -2474,7 +2668,7 @@
       </c>
     </row>
     <row r="4" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="A4" s="2">
+      <c r="A4" s="1">
         <v>3</v>
       </c>
       <c r="B4">
@@ -2499,7 +2693,7 @@
       </c>
     </row>
     <row r="5" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="A5" s="2">
+      <c r="A5" s="1">
         <v>4</v>
       </c>
       <c r="B5">
@@ -2524,7 +2718,7 @@
       </c>
     </row>
     <row r="6" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="A6" s="2">
+      <c r="A6" s="1">
         <v>5</v>
       </c>
       <c r="B6">
@@ -2549,7 +2743,7 @@
       </c>
     </row>
     <row r="7" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="A7" s="2">
+      <c r="A7" s="1">
         <v>6</v>
       </c>
       <c r="B7">
@@ -2574,7 +2768,7 @@
       </c>
     </row>
     <row r="8" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="A8" s="2">
+      <c r="A8" s="1">
         <v>7</v>
       </c>
       <c r="B8">
@@ -2599,7 +2793,7 @@
       </c>
     </row>
     <row r="9" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="A9" s="2">
+      <c r="A9" s="1">
         <v>8</v>
       </c>
       <c r="B9">
@@ -2624,7 +2818,7 @@
       </c>
     </row>
     <row r="10" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="A10" s="2">
+      <c r="A10" s="1">
         <v>9</v>
       </c>
       <c r="B10">
@@ -2649,7 +2843,7 @@
       </c>
     </row>
     <row r="11" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="A11" s="2">
+      <c r="A11" s="1">
         <v>10</v>
       </c>
       <c r="B11">
@@ -2674,7 +2868,7 @@
       </c>
     </row>
     <row r="12" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="A12" s="2">
+      <c r="A12" s="1">
         <v>11</v>
       </c>
       <c r="B12">
@@ -2699,7 +2893,7 @@
       </c>
     </row>
     <row r="13" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="A13" s="2">
+      <c r="A13" s="1">
         <v>12</v>
       </c>
       <c r="B13">
@@ -2724,7 +2918,7 @@
       </c>
     </row>
     <row r="14" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="A14" s="2">
+      <c r="A14" s="1">
         <v>13</v>
       </c>
       <c r="B14">
@@ -2749,7 +2943,7 @@
       </c>
     </row>
     <row r="15" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="A15" s="2">
+      <c r="A15" s="1">
         <v>14</v>
       </c>
       <c r="B15">
@@ -2774,7 +2968,7 @@
       </c>
     </row>
     <row r="16" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="A16" s="2">
+      <c r="A16" s="1">
         <v>15</v>
       </c>
       <c r="B16">
@@ -2799,7 +2993,7 @@
       </c>
     </row>
     <row r="17" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="A17" s="2">
+      <c r="A17" s="1">
         <v>16</v>
       </c>
       <c r="B17">
@@ -2824,7 +3018,7 @@
       </c>
     </row>
     <row r="18" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="A18" s="2">
+      <c r="A18" s="1">
         <v>17</v>
       </c>
       <c r="B18">
@@ -2849,7 +3043,7 @@
       </c>
     </row>
     <row r="19" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="A19" s="2">
+      <c r="A19" s="1">
         <v>18</v>
       </c>
       <c r="B19">
@@ -2874,7 +3068,7 @@
       </c>
     </row>
     <row r="20" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="A20" s="2">
+      <c r="A20" s="1">
         <v>19</v>
       </c>
       <c r="B20">
@@ -2899,7 +3093,7 @@
       </c>
     </row>
     <row r="21" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="A21" s="2">
+      <c r="A21" s="1">
         <v>20</v>
       </c>
       <c r="B21">
@@ -2924,7 +3118,7 @@
       </c>
     </row>
     <row r="22" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="A22" s="2">
+      <c r="A22" s="1">
         <v>21</v>
       </c>
       <c r="B22">
@@ -2949,7 +3143,7 @@
       </c>
     </row>
     <row r="23" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="A23" s="2">
+      <c r="A23" s="1">
         <v>22</v>
       </c>
       <c r="B23">
@@ -2974,7 +3168,7 @@
       </c>
     </row>
     <row r="24" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="A24" s="2">
+      <c r="A24" s="1">
         <v>23</v>
       </c>
       <c r="B24">
@@ -2999,7 +3193,7 @@
       </c>
     </row>
     <row r="25" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="A25" s="2">
+      <c r="A25" s="1">
         <v>24</v>
       </c>
       <c r="B25">
@@ -3024,7 +3218,7 @@
       </c>
     </row>
     <row r="26" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="A26" s="2">
+      <c r="A26" s="1">
         <v>25</v>
       </c>
       <c r="B26">
@@ -3049,7 +3243,7 @@
       </c>
     </row>
     <row r="27" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="A27" s="2">
+      <c r="A27" s="1">
         <v>26</v>
       </c>
       <c r="B27">
@@ -3074,7 +3268,7 @@
       </c>
     </row>
     <row r="28" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="A28" s="2">
+      <c r="A28" s="1">
         <v>27</v>
       </c>
       <c r="B28">
@@ -3099,7 +3293,7 @@
       </c>
     </row>
     <row r="29" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="A29" s="2">
+      <c r="A29" s="1">
         <v>28</v>
       </c>
       <c r="B29">
@@ -3124,7 +3318,7 @@
       </c>
     </row>
     <row r="30" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="A30" s="2">
+      <c r="A30" s="1">
         <v>29</v>
       </c>
       <c r="B30">
@@ -3149,7 +3343,7 @@
       </c>
     </row>
     <row r="31" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="A31" s="2">
+      <c r="A31" s="1">
         <v>30</v>
       </c>
       <c r="B31">
@@ -3174,7 +3368,7 @@
       </c>
     </row>
     <row r="32" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="A32" s="2">
+      <c r="A32" s="1">
         <v>31</v>
       </c>
       <c r="B32">
@@ -3199,7 +3393,7 @@
       </c>
     </row>
     <row r="33" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="A33" s="2">
+      <c r="A33" s="1">
         <v>32</v>
       </c>
       <c r="B33">
@@ -3224,7 +3418,7 @@
       </c>
     </row>
     <row r="34" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="A34" s="2">
+      <c r="A34" s="1">
         <v>33</v>
       </c>
       <c r="B34">
@@ -3249,7 +3443,7 @@
       </c>
     </row>
     <row r="35" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="A35" s="2">
+      <c r="A35" s="1">
         <v>34</v>
       </c>
       <c r="B35">
@@ -3274,7 +3468,7 @@
       </c>
     </row>
     <row r="36" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="A36" s="2">
+      <c r="A36" s="1">
         <v>35</v>
       </c>
       <c r="B36">

</xml_diff>